<commit_message>
Set FSPbPPT to 0
</commit_message>
<xml_diff>
--- a/InputData/fuels/FSPbPPT/Fuel Surcharge Perc by Power Plant Type.xlsx
+++ b/InputData/fuels/FSPbPPT/Fuel Surcharge Perc by Power Plant Type.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\fuels\FSPbPPT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\fuels\FSPbPPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65263F8A-FDBA-4D8E-81F2-4CDEE15290AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E68A24-8001-45EF-83F0-565A10AD0B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Source:</t>
   </si>
@@ -109,24 +109,6 @@
     <t>However, that variable is subscripted by All Fuels, not by Electricity Source (i.e., power plant type).</t>
   </si>
   <si>
-    <t>Peaking power plants, which only consume small amounts of fuel at irregular intervals, may face higher costs</t>
-  </si>
-  <si>
-    <t>per unit fuel than a power plant that purchases larger quantities of fuel at a steady rate.</t>
-  </si>
-  <si>
-    <t>but pay higher prices per unit of fuel purchased than those other plants.</t>
-  </si>
-  <si>
-    <t>This mostly applies to natural gas peaker plants and natural gas steam turbines, which buy the same fuel as</t>
-  </si>
-  <si>
-    <t>natural gas combined cycle plants, but face higher costs per unit fuel than natural gas combined cycle plants.</t>
-  </si>
-  <si>
-    <t>Therefore, it is necessary to apply a surcharge to plant types that use the same fuel type as other plants</t>
-  </si>
-  <si>
     <t>hard coal w CCS</t>
   </si>
   <si>
@@ -146,6 +128,9 @@
   </si>
   <si>
     <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>We are currently not using this surcharge for any plant types in the US model.</t>
   </si>
 </sst>
 </file>
@@ -239,7 +224,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -253,7 +238,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -580,33 +564,14 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="A19" s="1"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="A20" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -647,7 +612,7 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -727,7 +692,7 @@
         <v>8</v>
       </c>
       <c r="B13">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -772,57 +737,57 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="7">
+        <v>24</v>
+      </c>
+      <c r="B19">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="7">
+        <v>25</v>
+      </c>
+      <c r="B20">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="7">
+        <v>26</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="7">
+        <v>27</v>
+      </c>
+      <c r="B22">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>34</v>
-      </c>
-      <c r="B23" s="7">
+        <v>28</v>
+      </c>
+      <c r="B23">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="7">
+      <c r="A24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="7">
+      <c r="A25" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
         <v>0</v>
       </c>
     </row>

</xml_diff>